<commit_message>
La Prière : EAN attribués (garçon 9782919843251, fille 9782919843268) et retrait du tirage du dossier
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lapriere_kit/fiche-technique-matrice.xlsx
+++ b/lapriere_kit/fiche-technique-matrice.xlsx
@@ -679,7 +679,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -927,6 +927,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="22" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1548,7 +1551,11 @@
           <t>Éveil à l'islam pour les petits</t>
         </is>
       </c>
-      <c r="C2" s="92" t="n"/>
+      <c r="C2" s="109" t="inlineStr">
+        <is>
+          <t>9782919843251</t>
+        </is>
+      </c>
       <c r="D2" s="91" t="inlineStr">
         <is>
           <t>Le papa du petit Adam a décidé de lui apprendre la prière. Adam est impatient de savoir faire la prière comme son papa. Il apprend à faire ses ablutions dans le jardin, avec un seau d'eau, met sa plus belle tenue, déroule son tapis… et aujourd'hui, il a effectué sa première prière comme un grand !
@@ -1675,7 +1682,11 @@
           <t>Éveil à l'islam pour les petits</t>
         </is>
       </c>
-      <c r="C3" s="92" t="n"/>
+      <c r="C3" s="109" t="inlineStr">
+        <is>
+          <t>9782919843268</t>
+        </is>
+      </c>
       <c r="D3" s="91" t="inlineStr">
         <is>
           <t>La maman de la petite Sophia a décidé de lui apprendre la prière. Sophia est impatiente de savoir faire la prière comme sa maman. Elle apprend à faire ses ablutions dans la salle de bain, enfile une longue tenue de prière, déroule son tapis… et aujourd'hui, elle a effectué sa première prière comme une grande !
@@ -4209,7 +4220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4227,7 +4238,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="37" t="inlineStr">
         <is>
-          <t>Fiche technique remplie le 21/09/2026 pour les deux versions, avec les conventions de la matrice maison « Présentation des livres du BDouin ». Les cellules jaunes restent à renseigner.</t>
+          <t>Fiche technique remplie le 21/09/2026 pour les deux versions, avec les conventions de la matrice maison « Présentation des livres du BDouin ». EAN attribués le 22/09/2026 : garçon 9782919843251, fille 9782919843268 (feuille « isbn BDOUIN », lignes « Je m'éveille à l'Islam »).</t>
         </is>
       </c>
     </row>
@@ -4251,29 +4262,29 @@
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="101" t="inlineStr">
         <is>
-          <t>EAN</t>
+          <t>Nombre de pages</t>
         </is>
       </c>
       <c r="B5" s="37" t="inlineStr">
         <is>
-          <t>Aucun EAN attribué. Dans « isbn BDOUIN », les deux prochains libres de la plage 978-2-919843 sont 9782919843084 et 9782919843091 (08 et 09 ; 00 à 07, 17, 19 à 22 sont déjà pris).</t>
+          <t>Aucun PDF imprimeur. Repères maison : Walad découvre Médine 71 p., Mini Guide Salat 87 p.</t>
         </is>
       </c>
       <c r="C5" s="37" t="inlineStr">
         <is>
-          <t>Karim, à attribuer</t>
+          <t>Fiche technique IMAK</t>
         </is>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="101" t="inlineStr">
         <is>
-          <t>Nombre de pages</t>
+          <t>Épaisseur, largeur, hauteur</t>
         </is>
       </c>
       <c r="B6" s="37" t="inlineStr">
         <is>
-          <t>Aucun PDF imprimeur. Repères maison : Walad découvre Médine 71 p., Mini Guide Salat 87 p.</t>
+          <t>Le livre est carré. Le gabarit maison le plus proche est Walad découvre Médine : 21,4 × 22 cm, épaisseur 1,22 cm.</t>
         </is>
       </c>
       <c r="C6" s="37" t="inlineStr">
@@ -4285,12 +4296,12 @@
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="101" t="inlineStr">
         <is>
-          <t>Épaisseur, largeur, hauteur</t>
+          <t>Poids</t>
         </is>
       </c>
       <c r="B7" s="37" t="inlineStr">
         <is>
-          <t>Le livre est carré. Le gabarit maison le plus proche est Walad découvre Médine : 21,4 × 22 cm, épaisseur 1,22 cm.</t>
+          <t>Walad découvre Médine pèse 473 g, les Mini Guides 296 à 300 g.</t>
         </is>
       </c>
       <c r="C7" s="37" t="inlineStr">
@@ -4300,34 +4311,30 @@
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="101" t="inlineStr">
-        <is>
-          <t>Poids</t>
-        </is>
-      </c>
-      <c r="B8" s="37" t="inlineStr">
-        <is>
-          <t>Walad découvre Médine pèse 473 g, les Mini Guides 296 à 300 g.</t>
-        </is>
-      </c>
-      <c r="C8" s="37" t="inlineStr">
-        <is>
-          <t>Fiche technique IMAK</t>
-        </is>
-      </c>
+      <c r="A8" s="101" t="n"/>
+      <c r="B8" s="37" t="n"/>
+      <c r="C8" s="37" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="101" t="n"/>
+      <c r="A9" s="102" t="inlineStr">
+        <is>
+          <t>Repris de la matrice maison</t>
+        </is>
+      </c>
       <c r="B9" s="37" t="n"/>
       <c r="C9" s="37" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="102" t="inlineStr">
-        <is>
-          <t>Repris de la matrice maison</t>
-        </is>
-      </c>
-      <c r="B10" s="37" t="n"/>
+      <c r="A10" s="101" t="inlineStr">
+        <is>
+          <t>·</t>
+        </is>
+      </c>
+      <c r="B10" s="37" t="inlineStr">
+        <is>
+          <t>Auteur et illustrateur : Norédine Allam pour les deux, comme sur toutes les lignes de la matrice maison.</t>
+        </is>
+      </c>
       <c r="C10" s="37" t="n"/>
     </row>
     <row r="11" ht="28" customHeight="1">
@@ -4338,7 +4345,7 @@
       </c>
       <c r="B11" s="37" t="inlineStr">
         <is>
-          <t>Auteur et illustrateur : Norédine Allam pour les deux, comme sur toutes les lignes de la matrice maison.</t>
+          <t>Éditeur : « Bdouin », orthographe de la matrice maison.</t>
         </is>
       </c>
       <c r="C11" s="37" t="n"/>
@@ -4351,45 +4358,44 @@
       </c>
       <c r="B12" s="37" t="inlineStr">
         <is>
-          <t>Éditeur : « Bdouin », orthographe de la matrice maison.</t>
+          <t>Catégorie 40114 « Jeunesse » (sous Islam) : celle utilisée pour tous les titres BDouin, y compris les Mini Guides et Walad découvre Médine.</t>
         </is>
       </c>
       <c r="C12" s="37" t="n"/>
     </row>
     <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="101" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
       <c r="B13" s="37" t="inlineStr">
         <is>
-          <t>Catégorie 40114 « Jeunesse » (sous Islam) : celle utilisée pour tous les titres BDouin, y compris les Mini Guides et Walad découvre Médine.</t>
-        </is>
-      </c>
-      <c r="C13" s="37" t="n"/>
+          <t>Présentation « Livre relié » : la matrice maison dit « rigide » pour tous les albums ; « Livre relié » est le libellé de la liste Sofiadis.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="102" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
       <c r="B14" s="37" t="inlineStr">
         <is>
-          <t>Présentation « Livre relié » : la matrice maison dit « rigide » pour tous les albums ; « Livre relié » est le libellé de la liste Sofiadis.</t>
+          <t>Prix HT 9,48 € : 10 € TTC au taux 5,5 % (décision Karim du 21/09, les Mini Guides sont à 12 €).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="102" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
       <c r="B15" s="37" t="inlineStr">
         <is>
-          <t>Prix HT 9,48 € : 10 € TTC au taux 5,5 % (décision Karim du 21/09, les Mini Guides sont à 12 €).</t>
+          <t>Parution 01/10/2026 : estimation, le jour exact reste à fixer.</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4407,7 @@
       </c>
       <c r="B16" s="37" t="inlineStr">
         <is>
-          <t>Parution 01/10/2026 : estimation, le jour exact reste à fixer.</t>
+          <t>Désignation « La Prière - Version garçon / fille » : le titre seul ne distingue pas les deux articles.</t>
         </is>
       </c>
     </row>
@@ -4413,24 +4419,12 @@
       </c>
       <c r="B17" s="37" t="inlineStr">
         <is>
-          <t>Désignation « La Prière - Version garçon / fille » : le titre seul ne distingue pas les deux articles.</t>
+          <t>Colonnes Prix HT réservé, Fournisseur à Dilicom : laissées à Sofiadis.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>·</t>
-        </is>
-      </c>
-      <c r="B18" s="37" t="inlineStr">
-        <is>
-          <t>Colonnes Prix HT réservé, Fournisseur à Dilicom : laissées à Sofiadis.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="37" t="n"/>
+      <c r="B18" s="37" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
La Prière : désignation de référencement « Éveil à l'islam pour les petits "La Prière" - garçon / - fille »
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lapriere_kit/fiche-technique-matrice.xlsx
+++ b/lapriere_kit/fiche-technique-matrice.xlsx
@@ -1543,12 +1543,12 @@
     <row r="2" ht="110" customHeight="1">
       <c r="A2" s="91" t="inlineStr">
         <is>
-          <t>La Prière - Version garçon</t>
+          <t>Éveil à l'islam pour les petits "La Prière" - garçon</t>
         </is>
       </c>
       <c r="B2" s="91" t="inlineStr">
         <is>
-          <t>Éveil à l'islam pour les petits</t>
+          <t>La Prière</t>
         </is>
       </c>
       <c r="C2" s="109" t="inlineStr">
@@ -1674,12 +1674,12 @@
     <row r="3" ht="110" customHeight="1">
       <c r="A3" s="91" t="inlineStr">
         <is>
-          <t>La Prière - Version fille</t>
+          <t>Éveil à l'islam pour les petits "La Prière" - fille</t>
         </is>
       </c>
       <c r="B3" s="91" t="inlineStr">
         <is>
-          <t>Éveil à l'islam pour les petits</t>
+          <t>La Prière</t>
         </is>
       </c>
       <c r="C3" s="109" t="inlineStr">
@@ -4238,7 +4238,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="37" t="inlineStr">
         <is>
-          <t>Fiche technique remplie le 21/09/2026 pour les deux versions, avec les conventions de la matrice maison « Présentation des livres du BDouin ». EAN attribués le 22/09/2026 : garçon 9782919843251, fille 9782919843268 (feuille « isbn BDOUIN », lignes « Je m'éveille à l'Islam »).</t>
+          <t>Fiche technique remplie le 21/09/2026 pour les deux versions, avec les conventions de la matrice maison « Présentation des livres du BDouin ». EAN attribués le 22/09/2026 : garçon 9782919843251, fille 9782919843268 (feuille « isbn BDOUIN », lignes « Je m'éveille à l'Islam »). Désignation imposée par Karim le 22/09/2026 : « Éveil à l'islam pour les petits "La Prière" - garçon / - fille », pour que le titre se retrouve au référencement.</t>
         </is>
       </c>
     </row>

</xml_diff>